<commit_message>
feat: v2 - Excel upload + alerts system + batch fetching
</commit_message>
<xml_diff>
--- a/listing_price_tracker.xlsx
+++ b/listing_price_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://genmills-my.sharepoint.com/personal/joffray_dealberto_genmills_com/Documents/Desktop/Dossier Perso/Github/price_tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{3EF116D2-B036-48A6-81E5-9BA127B540D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8_{6094A151-DE15-4151-90D1-78211AE6B67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{83928C85-9E9A-4A80-BD61-F1AA46A075AC}"/>
+    <workbookView minimized="1" xWindow="450" yWindow="450" windowWidth="19180" windowHeight="11260" activeTab="1" xr2:uid="{83928C85-9E9A-4A80-BD61-F1AA46A075AC}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -6228,6 +6228,7 @@
   <dimension ref="A1:L115"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="16.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.6328125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.7265625" bestFit="1" customWidth="1"/>

</xml_diff>